<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-17 14:31 UTC
</commit_message>
<xml_diff>
--- a/data/50001559 - FERROVIAL.xlsx
+++ b/data/50001559 - FERROVIAL.xlsx
@@ -2691,7 +2691,7 @@
       </c>
       <c r="C17" s="9"/>
       <c r="D17" s="8">
-        <v>46182.62896958333</v>
+        <v>46190.51816748842</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>76</v>
@@ -4974,7 +4974,7 @@
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="5">
-        <v>46184.198145</v>
+        <v>46190.51911810185</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>202</v>
@@ -5249,7 +5249,7 @@
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46182.627335625</v>
+        <v>46190.519194259265</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>218</v>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46182.62733162037</v>
+        <v>46190.51933267361</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>99</v>

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-17 17:29 UTC
</commit_message>
<xml_diff>
--- a/data/50001559 - FERROVIAL.xlsx
+++ b/data/50001559 - FERROVIAL.xlsx
@@ -3875,7 +3875,7 @@
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46190.67767923611</v>
+        <v>46190.72156443287</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>142</v>
@@ -4962,7 +4962,7 @@
       </c>
       <c r="C55" s="10"/>
       <c r="D55" s="9">
-        <v>46181.77194856481</v>
+        <v>46190.70825689815</v>
       </c>
       <c r="E55" s="10" t="s">
         <v>200</v>
@@ -5007,9 +5007,11 @@
       <c r="B56" s="5">
         <v>46181.60908480324</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46190.708245752314</v>
+      </c>
       <c r="D56" s="5">
-        <v>46190.675336354165</v>
+        <v>46190.708260555555</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>203</v>
@@ -5057,10 +5059,10 @@
         <v>207</v>
       </c>
       <c r="T56" s="6">
-        <v>0</v>
-      </c>
-      <c r="U56" s="11" t="s">
-        <v>57</v>
+        <v>1</v>
+      </c>
+      <c r="U56" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -5070,9 +5072,11 @@
       <c r="B57" s="9">
         <v>46181.60908915509</v>
       </c>
-      <c r="C57" s="10"/>
+      <c r="C57" s="9">
+        <v>46190.70821236111</v>
+      </c>
       <c r="D57" s="9">
-        <v>46190.677475335644</v>
+        <v>46190.70821390046</v>
       </c>
       <c r="E57" s="10" t="s">
         <v>209</v>
@@ -5123,9 +5127,11 @@
       <c r="B58" s="5">
         <v>46181.60909384259</v>
       </c>
-      <c r="C58" s="6"/>
+      <c r="C58" s="5">
+        <v>46190.70822138889</v>
+      </c>
       <c r="D58" s="5">
-        <v>46190.677476377314</v>
+        <v>46190.7082228125</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>212</v>
@@ -5176,9 +5182,11 @@
       <c r="B59" s="9">
         <v>46181.61221741898</v>
       </c>
-      <c r="C59" s="10"/>
+      <c r="C59" s="9">
+        <v>46190.70822601852</v>
+      </c>
       <c r="D59" s="9">
-        <v>46190.677470173614</v>
+        <v>46190.708227337964</v>
       </c>
       <c r="E59" s="10" t="s">
         <v>215</v>
@@ -5229,9 +5237,11 @@
       <c r="B60" s="5">
         <v>46181.612357199076</v>
       </c>
-      <c r="C60" s="6"/>
+      <c r="C60" s="5">
+        <v>46190.70823167824</v>
+      </c>
       <c r="D60" s="5">
-        <v>46190.677471469906</v>
+        <v>46190.708233321755</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>217</v>
@@ -5345,7 +5355,7 @@
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="5">
-        <v>46182.632599652774</v>
+        <v>46190.70821725695</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>209</v>
@@ -5398,7 +5408,7 @@
       </c>
       <c r="C63" s="10"/>
       <c r="D63" s="9">
-        <v>46182.632596678246</v>
+        <v>46190.70822666667</v>
       </c>
       <c r="E63" s="10" t="s">
         <v>212</v>
@@ -5449,9 +5459,11 @@
       <c r="B64" s="5">
         <v>46181.61393570602</v>
       </c>
-      <c r="C64" s="6"/>
+      <c r="C64" s="5">
+        <v>46190.70842026621</v>
+      </c>
       <c r="D64" s="5">
-        <v>46182.63259350695</v>
+        <v>46190.70842170139</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>215</v>
@@ -5502,9 +5514,11 @@
       <c r="B65" s="9">
         <v>46181.61396929398</v>
       </c>
-      <c r="C65" s="10"/>
+      <c r="C65" s="9">
+        <v>46190.70842520833</v>
+      </c>
       <c r="D65" s="9">
-        <v>46182.63259271991</v>
+        <v>46190.708426550926</v>
       </c>
       <c r="E65" s="10" t="s">
         <v>217</v>
@@ -5720,9 +5734,11 @@
       <c r="B69" s="9">
         <v>46181.614119606485</v>
       </c>
-      <c r="C69" s="10"/>
+      <c r="C69" s="9">
+        <v>46190.72172383102</v>
+      </c>
       <c r="D69" s="9">
-        <v>46182.63268149305</v>
+        <v>46190.721725358795</v>
       </c>
       <c r="E69" s="10" t="s">
         <v>215</v>
@@ -5771,9 +5787,11 @@
       <c r="B70" s="5">
         <v>46181.61419627315</v>
       </c>
-      <c r="C70" s="6"/>
+      <c r="C70" s="5">
+        <v>46190.72172868055</v>
+      </c>
       <c r="D70" s="5">
-        <v>46182.63267761574</v>
+        <v>46190.7217299537</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>217</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-23 16:01 UTC
</commit_message>
<xml_diff>
--- a/data/50001559 - FERROVIAL.xlsx
+++ b/data/50001559 - FERROVIAL.xlsx
@@ -346,25 +346,25 @@
     <t>Generación OC materiales corte Laser ot 4342 -4344,Propuesta compras:</t>
   </si>
   <si>
+    <t>1215506984624491</t>
+  </si>
+  <si>
+    <t>Propuesta Corte plasma  ot 4347</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generación OC Corte Plasma  ot 4342 -4344 </t>
+  </si>
+  <si>
+    <t>1215506992580924</t>
+  </si>
+  <si>
+    <t>Propuesta Mecanizado ot 4347</t>
+  </si>
+  <si>
+    <t>Generación OC Mecanizado ot 4342 -4344</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1215506984624491</t>
-  </si>
-  <si>
-    <t>Propuesta Corte plasma  ot 4347</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generación OC Corte Plasma  ot 4342 -4344 </t>
-  </si>
-  <si>
-    <t>1215506992580924</t>
-  </si>
-  <si>
-    <t>Propuesta Mecanizado ot 4347</t>
-  </si>
-  <si>
-    <t>Generación OC Mecanizado ot 4342 -4344</t>
   </si>
   <si>
     <t>1215506992580936</t>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="5">
-        <v>46190.67771045139</v>
+        <v>46196.65857491898</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>79</v>
@@ -2924,9 +2924,11 @@
       <c r="B22" s="5">
         <v>46181.60888054398</v>
       </c>
-      <c r="C22" s="6"/>
+      <c r="C22" s="5">
+        <v>46196.658568541665</v>
+      </c>
       <c r="D22" s="5">
-        <v>46191.67365563658</v>
+        <v>46196.65858296296</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>92</v>
@@ -2974,25 +2976,27 @@
         <v>32</v>
       </c>
       <c r="T22" s="6">
-        <v>0</v>
-      </c>
-      <c r="U22" s="12" t="s">
-        <v>97</v>
+        <v>1</v>
+      </c>
+      <c r="U22" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B23" s="8">
         <v>46181.60888559028</v>
       </c>
-      <c r="C23" s="9"/>
+      <c r="C23" s="8">
+        <v>46196.65883074074</v>
+      </c>
       <c r="D23" s="8">
-        <v>46191.67366451389</v>
+        <v>46196.658845625</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
@@ -3025,7 +3029,7 @@
         <v>95</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="Q23" s="8">
         <v>46248</v>
@@ -3037,15 +3041,15 @@
         <v>32</v>
       </c>
       <c r="T23" s="9">
-        <v>0</v>
-      </c>
-      <c r="U23" s="12" t="s">
-        <v>97</v>
+        <v>1</v>
+      </c>
+      <c r="U23" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B24" s="5">
         <v>46181.60888961806</v>
@@ -3055,7 +3059,7 @@
         <v>46191.67367153935</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
@@ -3088,7 +3092,7 @@
         <v>95</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="Q24" s="5">
         <v>46248</v>
@@ -3103,7 +3107,7 @@
         <v>0</v>
       </c>
       <c r="U24" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
@@ -3166,7 +3170,7 @@
         <v>0</v>
       </c>
       <c r="U25" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
@@ -3341,7 +3345,7 @@
         <v>0</v>
       </c>
       <c r="U28" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3404,7 +3408,7 @@
         <v>0</v>
       </c>
       <c r="U29" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3760,7 +3764,7 @@
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="5">
-        <v>46182.62676782407</v>
+        <v>46196.65857439815</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>136</v>
@@ -3941,10 +3945,10 @@
       </c>
       <c r="C39" s="9"/>
       <c r="D39" s="8">
-        <v>46182.626871608794</v>
+        <v>46196.65883732639</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>26</v>
@@ -3974,7 +3978,7 @@
         <v>142</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>145</v>
@@ -4027,7 +4031,7 @@
         <v>142</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>148</v>
@@ -4335,7 +4339,7 @@
         <v>46182.62720454861</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
@@ -4365,7 +4369,7 @@
         <v>164</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>167</v>
@@ -4418,7 +4422,7 @@
         <v>164</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="P47" s="9" t="s">
         <v>170</v>
@@ -4475,7 +4479,7 @@
       <c r="S48" s="6"/>
       <c r="T48" s="6"/>
       <c r="U48" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
@@ -7057,7 +7061,7 @@
         <v>0</v>
       </c>
       <c r="U94" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="95" spans="1:21" x14ac:dyDescent="0.25">
@@ -7120,7 +7124,7 @@
         <v>0</v>
       </c>
       <c r="U95" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="96" spans="1:21" x14ac:dyDescent="0.25">
@@ -7183,7 +7187,7 @@
         <v>0</v>
       </c>
       <c r="U96" s="12" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
     </row>
     <row r="97" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
KPI actualizado 2026-07-13 15:50 UTC
</commit_message>
<xml_diff>
--- a/data/50001559 - FERROVIAL.xlsx
+++ b/data/50001559 - FERROVIAL.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1818" uniqueCount="396">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1819" uniqueCount="396">
   <si>
     <t>50001559 - FERROVIAL</t>
   </si>
@@ -5598,9 +5598,11 @@
       <c r="B67" s="8">
         <v>46181.60918671296</v>
       </c>
-      <c r="C67" s="9"/>
+      <c r="C67" s="8">
+        <v>46216.64128039352</v>
+      </c>
       <c r="D67" s="8">
-        <v>46213.569374502316</v>
+        <v>46216.64129429398</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>216</v>
@@ -5635,8 +5637,12 @@
       <c r="Q67" s="9"/>
       <c r="R67" s="9"/>
       <c r="S67" s="9"/>
-      <c r="T67" s="9"/>
-      <c r="U67" s="9"/>
+      <c r="T67" s="9">
+        <v>1</v>
+      </c>
+      <c r="U67" s="10" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="4" t="s">
@@ -5710,9 +5716,11 @@
       <c r="B69" s="8">
         <v>46181.609201921296</v>
       </c>
-      <c r="C69" s="9"/>
+      <c r="C69" s="8">
+        <v>46216.6412221875</v>
+      </c>
       <c r="D69" s="8">
-        <v>46213.56940306713</v>
+        <v>46216.641245011575</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>224</v>
@@ -5760,10 +5768,10 @@
         <v>32</v>
       </c>
       <c r="T69" s="9">
-        <v>0</v>
-      </c>
-      <c r="U69" s="12" t="s">
-        <v>121</v>
+        <v>1</v>
+      </c>
+      <c r="U69" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -5838,9 +5846,11 @@
       <c r="B71" s="8">
         <v>46181.609212870375</v>
       </c>
-      <c r="C71" s="9"/>
+      <c r="C71" s="8">
+        <v>46216.641230636575</v>
+      </c>
       <c r="D71" s="8">
-        <v>46213.569403009256</v>
+        <v>46216.641249629625</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>231</v>
@@ -5888,10 +5898,10 @@
         <v>32</v>
       </c>
       <c r="T71" s="9">
-        <v>0</v>
-      </c>
-      <c r="U71" s="12" t="s">
-        <v>121</v>
+        <v>1</v>
+      </c>
+      <c r="U71" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="72" spans="1:21" x14ac:dyDescent="0.25">
@@ -5966,9 +5976,11 @@
       <c r="B73" s="8">
         <v>46181.60922180556</v>
       </c>
-      <c r="C73" s="9"/>
+      <c r="C73" s="8">
+        <v>46216.64126351852</v>
+      </c>
       <c r="D73" s="8">
-        <v>46213.56941956018</v>
+        <v>46216.641280717595</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>235</v>
@@ -6016,10 +6028,10 @@
         <v>32</v>
       </c>
       <c r="T73" s="9">
-        <v>0</v>
-      </c>
-      <c r="U73" s="12" t="s">
-        <v>121</v>
+        <v>1</v>
+      </c>
+      <c r="U73" s="10" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -6141,7 +6153,7 @@
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46204.88313940972</v>
+        <v>46216.641273009256</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>182</v>
@@ -6194,7 +6206,7 @@
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46182.63598342593</v>
+        <v>46216.64127412037</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>182</v>
@@ -6247,7 +6259,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46182.63598072917</v>
+        <v>46216.64126927083</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>187</v>
@@ -6300,7 +6312,7 @@
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46182.63597787037</v>
+        <v>46216.64127059028</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>190</v>
@@ -6353,7 +6365,7 @@
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46182.635973807875</v>
+        <v>46216.641271817134</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>192</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-28 21:21 UTC
</commit_message>
<xml_diff>
--- a/data/50001559 - FERROVIAL.xlsx
+++ b/data/50001559 - FERROVIAL.xlsx
@@ -6061,7 +6061,7 @@
         <v>46225.80622738426</v>
       </c>
       <c r="D75" s="8">
-        <v>46231.56036584491</v>
+        <v>46231.65309723379</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>240</v>
@@ -8349,7 +8349,7 @@
       </c>
       <c r="C115" s="9"/>
       <c r="D115" s="8">
-        <v>46230.85274487268</v>
+        <v>46231.862803634256</v>
       </c>
       <c r="E115" s="9" t="s">
         <v>186</v>
@@ -8455,7 +8455,7 @@
       </c>
       <c r="C117" s="9"/>
       <c r="D117" s="8">
-        <v>46230.85292063658</v>
+        <v>46231.86380424768</v>
       </c>
       <c r="E117" s="9" t="s">
         <v>333</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-22 16:39 Chile
</commit_message>
<xml_diff>
--- a/data/50001559 - FERROVIAL.xlsx
+++ b/data/50001559 - FERROVIAL.xlsx
@@ -1828,7 +1828,7 @@
         <v>46190.67646162037</v>
       </c>
       <c r="D4" s="5">
-        <v>46233.51851459491</v>
+        <v>46256.760763495375</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -5107,7 +5107,7 @@
         <v>46191.54538693287</v>
       </c>
       <c r="D59" s="8">
-        <v>46248.18694645833</v>
+        <v>46256.76246777778</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>96</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-23 09:44 Chile
</commit_message>
<xml_diff>
--- a/data/50001559 - FERROVIAL.xlsx
+++ b/data/50001559 - FERROVIAL.xlsx
@@ -1828,7 +1828,7 @@
         <v>46190.67646162037</v>
       </c>
       <c r="D4" s="5">
-        <v>46256.760763495375</v>
+        <v>46257.25799886574</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -5382,7 +5382,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46212.622826203704</v>
+        <v>46256.986112349536</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>208</v>
@@ -9376,7 +9376,7 @@
       </c>
       <c r="C134" s="6"/>
       <c r="D134" s="5">
-        <v>46253.64385789352</v>
+        <v>46257.009018275465</v>
       </c>
       <c r="E134" s="6" t="s">
         <v>355</v>

</xml_diff>